<commit_message>
fix unknown detection and fix notebook
</commit_message>
<xml_diff>
--- a/src/result/lfw/comparison_no_svd.xlsx
+++ b/src/result/lfw/comparison_no_svd.xlsx
@@ -457,7 +457,7 @@
         <v>0.5906855625219409</v>
       </c>
       <c r="E2" t="n">
-        <v>2.848417997360229</v>
+        <v>1.672689199447632</v>
       </c>
     </row>
     <row r="3">
@@ -474,7 +474,7 @@
         <v>0.82633665194647</v>
       </c>
       <c r="E3" t="n">
-        <v>1.474628210067749</v>
+        <v>1.400212287902832</v>
       </c>
     </row>
     <row r="4">
@@ -491,7 +491,7 @@
         <v>0.8176635612896228</v>
       </c>
       <c r="E4" t="n">
-        <v>3.06232476234436</v>
+        <v>3.069623708724976</v>
       </c>
     </row>
   </sheetData>

</xml_diff>